<commit_message>
Add paper-ready robustness analysis and controlled Q4 comparison
</commit_message>
<xml_diff>
--- a/outputs/q1/result1.xlsx
+++ b/outputs/q1/result1.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计划购电量" sheetId="1" r:id="R90363054558847f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="充放电量" sheetId="2" r:id="R2d7bcb6e16e0416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计划购电量" sheetId="1" r:id="R457882679b9c4009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="充放电量" sheetId="2" r:id="Rd8f57ea06fa840f5"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>